<commit_message>
updated the  readme and the overview page
</commit_message>
<xml_diff>
--- a/quarto/data/RLE index scores bootstrap.xlsx
+++ b/quarto/data/RLE index scores bootstrap.xlsx
@@ -415,7 +415,7 @@
         <v>0.8909090909090909</v>
       </c>
       <c r="F2">
-        <v>0.8136363636363636</v>
+        <v>0.8090909090909091</v>
       </c>
       <c r="G2">
         <v>0.9590909090909091</v>
@@ -445,7 +445,7 @@
         <v>0.8545454545454545</v>
       </c>
       <c r="F3">
-        <v>0.7636363636363637</v>
+        <v>0.759090909090909</v>
       </c>
       <c r="G3">
         <v>0.9363636363636364</v>
@@ -505,7 +505,7 @@
         <v>0.8545454545454545</v>
       </c>
       <c r="F5">
-        <v>0.759090909090909</v>
+        <v>0.7636363636363637</v>
       </c>
       <c r="G5">
         <v>0.9363636363636364</v>
@@ -535,7 +535,7 @@
         <v>0.8555555555555556</v>
       </c>
       <c r="F6">
-        <v>0.7111111111111111</v>
+        <v>0.7222222222222222</v>
       </c>
       <c r="G6">
         <v>0.9666666666666667</v>
@@ -565,10 +565,10 @@
         <v>0.8111111111111111</v>
       </c>
       <c r="F7">
-        <v>0.6555555555555556</v>
+        <v>0.6666666666666667</v>
       </c>
       <c r="G7">
-        <v>0.9555555555555556</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -625,7 +625,7 @@
         <v>0.8111111111111111</v>
       </c>
       <c r="F9">
-        <v>0.6663888888888891</v>
+        <v>0.6666666666666667</v>
       </c>
       <c r="G9">
         <v>0.9333333333333333</v>
@@ -655,7 +655,7 @@
         <v>0.9066666666666666</v>
       </c>
       <c r="F10">
-        <v>0.76</v>
+        <v>0.7733333333333333</v>
       </c>
       <c r="G10">
         <v>1</v>
@@ -898,7 +898,7 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="G18">
-        <v>0.6952380952380952</v>
+        <v>0.6968253968253968</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>0.5523809523809524</v>
       </c>
       <c r="G19">
-        <v>0.680952380952381</v>
+        <v>0.6825396825396826</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -955,10 +955,10 @@
         <v>0.6174603174603175</v>
       </c>
       <c r="F20">
-        <v>0.5523809523809524</v>
+        <v>0.5507936507936508</v>
       </c>
       <c r="G20">
-        <v>0.6825396825396826</v>
+        <v>0.6841269841269841</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -985,7 +985,7 @@
         <v>0.6174603174603175</v>
       </c>
       <c r="F21">
-        <v>0.5523809523809524</v>
+        <v>0.553968253968254</v>
       </c>
       <c r="G21">
         <v>0.680952380952381</v>
@@ -1045,10 +1045,10 @@
         <v>0.8191780821917808</v>
       </c>
       <c r="F23">
-        <v>0.7534246575342466</v>
+        <v>0.7506849315068493</v>
       </c>
       <c r="G23">
-        <v>0.8794520547945206</v>
+        <v>0.8821917808219178</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1078,7 +1078,7 @@
         <v>0.7561643835616438</v>
       </c>
       <c r="G24">
-        <v>0.8821917808219178</v>
+        <v>0.8794520547945206</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1408,7 +1408,7 @@
         <v>0.8361702127659575</v>
       </c>
       <c r="G35">
-        <v>0.9340425531914893</v>
+        <v>0.9319148936170213</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -1435,10 +1435,10 @@
         <v>0.874468085106383</v>
       </c>
       <c r="F36">
-        <v>0.8212765957446808</v>
+        <v>0.823404255319149</v>
       </c>
       <c r="G36">
-        <v>0.9234042553191489</v>
+        <v>0.9212765957446809</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -1465,7 +1465,7 @@
         <v>0.874468085106383</v>
       </c>
       <c r="F37">
-        <v>0.821223404255319</v>
+        <v>0.8212765957446808</v>
       </c>
       <c r="G37">
         <v>0.9234042553191489</v>
@@ -1495,7 +1495,7 @@
         <v>0.93125</v>
       </c>
       <c r="F38">
-        <v>0.875</v>
+        <v>0.871875</v>
       </c>
       <c r="G38">
         <v>0.978125</v>
@@ -1525,7 +1525,7 @@
         <v>0.91875</v>
       </c>
       <c r="F39">
-        <v>0.85625</v>
+        <v>0.859375</v>
       </c>
       <c r="G39">
         <v>0.96875</v>
@@ -1555,10 +1555,10 @@
         <v>0.91875</v>
       </c>
       <c r="F40">
-        <v>0.85625</v>
+        <v>0.8592968750000001</v>
       </c>
       <c r="G40">
-        <v>0.975</v>
+        <v>0.96875</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -1588,7 +1588,7 @@
         <v>0.85625</v>
       </c>
       <c r="G41">
-        <v>0.96875</v>
+        <v>0.975</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>0.770194384449244</v>
       </c>
       <c r="G43">
-        <v>0.8267818574514039</v>
+        <v>0.8272138228941684</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -1660,10 +1660,10 @@
         <v>0.7961123110151188</v>
       </c>
       <c r="F44">
-        <v>0.767170626349892</v>
+        <v>0.7676025917926566</v>
       </c>
       <c r="G44">
-        <v>0.8241900647948164</v>
+        <v>0.8250647948164145</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -1688,7 +1688,7 @@
         <v>0.7654427645788338</v>
       </c>
       <c r="G45">
-        <v>0.8215982721382289</v>
+        <v>0.8224622030237581</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
updated the email address in the overview page
</commit_message>
<xml_diff>
--- a/quarto/data/RLE index scores bootstrap.xlsx
+++ b/quarto/data/RLE index scores bootstrap.xlsx
@@ -415,7 +415,7 @@
         <v>0.8909090909090909</v>
       </c>
       <c r="F2">
-        <v>0.8090909090909091</v>
+        <v>0.8136363636363636</v>
       </c>
       <c r="G2">
         <v>0.9590909090909091</v>
@@ -445,7 +445,7 @@
         <v>0.8545454545454545</v>
       </c>
       <c r="F3">
-        <v>0.759090909090909</v>
+        <v>0.7636363636363637</v>
       </c>
       <c r="G3">
         <v>0.9363636363636364</v>
@@ -565,7 +565,7 @@
         <v>0.8111111111111111</v>
       </c>
       <c r="F7">
-        <v>0.6666666666666667</v>
+        <v>0.6555555555555556</v>
       </c>
       <c r="G7">
         <v>0.9333333333333333</v>
@@ -655,7 +655,7 @@
         <v>0.9066666666666666</v>
       </c>
       <c r="F10">
-        <v>0.7733333333333333</v>
+        <v>0.76</v>
       </c>
       <c r="G10">
         <v>1</v>
@@ -895,10 +895,10 @@
         <v>0.6333333333333333</v>
       </c>
       <c r="F18">
-        <v>0.5714285714285714</v>
+        <v>0.5682539682539682</v>
       </c>
       <c r="G18">
-        <v>0.6968253968253968</v>
+        <v>0.6984126984126984</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -925,7 +925,7 @@
         <v>0.6174603174603175</v>
       </c>
       <c r="F19">
-        <v>0.5523809523809524</v>
+        <v>0.553968253968254</v>
       </c>
       <c r="G19">
         <v>0.6825396825396826</v>
@@ -955,7 +955,7 @@
         <v>0.6174603174603175</v>
       </c>
       <c r="F20">
-        <v>0.5507936507936508</v>
+        <v>0.553968253968254</v>
       </c>
       <c r="G20">
         <v>0.6841269841269841</v>
@@ -985,7 +985,7 @@
         <v>0.6174603174603175</v>
       </c>
       <c r="F21">
-        <v>0.553968253968254</v>
+        <v>0.5523809523809524</v>
       </c>
       <c r="G21">
         <v>0.680952380952381</v>
@@ -1015,7 +1015,7 @@
         <v>0.8465753424657534</v>
       </c>
       <c r="F22">
-        <v>0.7890410958904109</v>
+        <v>0.7863013698630137</v>
       </c>
       <c r="G22">
         <v>0.9013698630136986</v>
@@ -1045,7 +1045,7 @@
         <v>0.8191780821917808</v>
       </c>
       <c r="F23">
-        <v>0.7506849315068493</v>
+        <v>0.7534246575342466</v>
       </c>
       <c r="G23">
         <v>0.8821917808219178</v>
@@ -1075,7 +1075,7 @@
         <v>0.8191780821917808</v>
       </c>
       <c r="F24">
-        <v>0.7561643835616438</v>
+        <v>0.7534246575342466</v>
       </c>
       <c r="G24">
         <v>0.8794520547945206</v>
@@ -1105,10 +1105,10 @@
         <v>0.8082191780821918</v>
       </c>
       <c r="F25">
-        <v>0.7424657534246575</v>
+        <v>0.7397260273972603</v>
       </c>
       <c r="G25">
-        <v>0.8712328767123287</v>
+        <v>0.873972602739726</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1408,7 +1408,7 @@
         <v>0.8361702127659575</v>
       </c>
       <c r="G35">
-        <v>0.9319148936170213</v>
+        <v>0.9340425531914893</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -1435,10 +1435,10 @@
         <v>0.874468085106383</v>
       </c>
       <c r="F36">
-        <v>0.823404255319149</v>
+        <v>0.8212765957446808</v>
       </c>
       <c r="G36">
-        <v>0.9212765957446809</v>
+        <v>0.9234042553191489</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -1585,10 +1585,10 @@
         <v>0.91875</v>
       </c>
       <c r="F41">
-        <v>0.85625</v>
+        <v>0.8561718749999999</v>
       </c>
       <c r="G41">
-        <v>0.975</v>
+        <v>0.971875</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -1610,10 +1610,10 @@
         <v>0.8215982721382289</v>
       </c>
       <c r="F42">
-        <v>0.7935205183585313</v>
+        <v>0.7939524838012959</v>
       </c>
       <c r="G42">
-        <v>0.8483801295896328</v>
+        <v>0.849244060475162</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -1635,10 +1635,10 @@
         <v>0.7987041036717063</v>
       </c>
       <c r="F43">
-        <v>0.770194384449244</v>
+        <v>0.7688984881209503</v>
       </c>
       <c r="G43">
-        <v>0.8272138228941684</v>
+        <v>0.8272246220302375</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -1660,10 +1660,10 @@
         <v>0.7961123110151188</v>
       </c>
       <c r="F44">
-        <v>0.7676025917926566</v>
+        <v>0.7663066954643629</v>
       </c>
       <c r="G44">
-        <v>0.8250647948164145</v>
+        <v>0.824622030237581</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
created a csv of a consolidated RLE assessments
</commit_message>
<xml_diff>
--- a/quarto/data/RLE index scores bootstrap.xlsx
+++ b/quarto/data/RLE index scores bootstrap.xlsx
@@ -415,10 +415,10 @@
         <v>0.8909090909090909</v>
       </c>
       <c r="F2">
-        <v>0.8136363636363636</v>
+        <v>0.8089772727272727</v>
       </c>
       <c r="G2">
-        <v>0.9590909090909091</v>
+        <v>0.9636363636363636</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -445,10 +445,10 @@
         <v>0.8545454545454545</v>
       </c>
       <c r="F3">
-        <v>0.7636363636363637</v>
+        <v>0.759090909090909</v>
       </c>
       <c r="G3">
-        <v>0.9363636363636364</v>
+        <v>0.9318181818181819</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -505,7 +505,7 @@
         <v>0.8545454545454545</v>
       </c>
       <c r="F5">
-        <v>0.7636363636363637</v>
+        <v>0.7635227272727273</v>
       </c>
       <c r="G5">
         <v>0.9363636363636364</v>
@@ -565,7 +565,7 @@
         <v>0.8111111111111111</v>
       </c>
       <c r="F7">
-        <v>0.6555555555555556</v>
+        <v>0.6663888888888891</v>
       </c>
       <c r="G7">
         <v>0.9333333333333333</v>
@@ -595,10 +595,10 @@
         <v>0.8111111111111111</v>
       </c>
       <c r="F8">
-        <v>0.6555555555555556</v>
+        <v>0.6666666666666667</v>
       </c>
       <c r="G8">
-        <v>0.9333333333333333</v>
+        <v>0.9338888888888808</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
         <v>0.5682539682539682</v>
       </c>
       <c r="G18">
-        <v>0.6984126984126984</v>
+        <v>0.6936507936507936</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -925,10 +925,10 @@
         <v>0.6174603174603175</v>
       </c>
       <c r="F19">
-        <v>0.553968253968254</v>
+        <v>0.5523809523809524</v>
       </c>
       <c r="G19">
-        <v>0.6825396825396826</v>
+        <v>0.680952380952381</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -955,10 +955,10 @@
         <v>0.6174603174603175</v>
       </c>
       <c r="F20">
-        <v>0.553968253968254</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="G20">
-        <v>0.6841269841269841</v>
+        <v>0.680952380952381</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -988,7 +988,7 @@
         <v>0.5523809523809524</v>
       </c>
       <c r="G21">
-        <v>0.680952380952381</v>
+        <v>0.6793650793650794</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
         <v>0.7863013698630137</v>
       </c>
       <c r="G22">
-        <v>0.9013698630136986</v>
+        <v>0.904109589041096</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
         <v>0.7534246575342466</v>
       </c>
       <c r="G23">
-        <v>0.8821917808219178</v>
+        <v>0.8794520547945206</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1078,7 +1078,7 @@
         <v>0.7534246575342466</v>
       </c>
       <c r="G24">
-        <v>0.8794520547945206</v>
+        <v>0.8795205479452045</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1105,10 +1105,10 @@
         <v>0.8082191780821918</v>
       </c>
       <c r="F25">
-        <v>0.7397260273972603</v>
+        <v>0.7424657534246575</v>
       </c>
       <c r="G25">
-        <v>0.873972602739726</v>
+        <v>0.8712328767123287</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
         <v>0.8617021276595744</v>
       </c>
       <c r="G34">
-        <v>0.951063829787234</v>
+        <v>0.948936170212766</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -1408,7 +1408,7 @@
         <v>0.8361702127659575</v>
       </c>
       <c r="G35">
-        <v>0.9340425531914893</v>
+        <v>0.9319148936170213</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -1435,7 +1435,7 @@
         <v>0.874468085106383</v>
       </c>
       <c r="F36">
-        <v>0.8212765957446808</v>
+        <v>0.823404255319149</v>
       </c>
       <c r="G36">
         <v>0.9234042553191489</v>
@@ -1465,7 +1465,7 @@
         <v>0.874468085106383</v>
       </c>
       <c r="F37">
-        <v>0.8212765957446808</v>
+        <v>0.823404255319149</v>
       </c>
       <c r="G37">
         <v>0.9234042553191489</v>
@@ -1495,7 +1495,7 @@
         <v>0.93125</v>
       </c>
       <c r="F38">
-        <v>0.871875</v>
+        <v>0.875</v>
       </c>
       <c r="G38">
         <v>0.978125</v>
@@ -1525,7 +1525,7 @@
         <v>0.91875</v>
       </c>
       <c r="F39">
-        <v>0.859375</v>
+        <v>0.85625</v>
       </c>
       <c r="G39">
         <v>0.96875</v>
@@ -1555,7 +1555,7 @@
         <v>0.91875</v>
       </c>
       <c r="F40">
-        <v>0.8592968750000001</v>
+        <v>0.859375</v>
       </c>
       <c r="G40">
         <v>0.96875</v>
@@ -1585,10 +1585,10 @@
         <v>0.91875</v>
       </c>
       <c r="F41">
-        <v>0.8561718749999999</v>
+        <v>0.85625</v>
       </c>
       <c r="G41">
-        <v>0.971875</v>
+        <v>0.96875</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -1610,10 +1610,10 @@
         <v>0.8215982721382289</v>
       </c>
       <c r="F42">
-        <v>0.7939524838012959</v>
+        <v>0.7930885529157667</v>
       </c>
       <c r="G42">
-        <v>0.849244060475162</v>
+        <v>0.8483801295896328</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -1635,10 +1635,10 @@
         <v>0.7987041036717063</v>
       </c>
       <c r="F43">
-        <v>0.7688984881209503</v>
+        <v>0.7693304535637149</v>
       </c>
       <c r="G43">
-        <v>0.8272246220302375</v>
+        <v>0.8267818574514039</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -1660,10 +1660,10 @@
         <v>0.7961123110151188</v>
       </c>
       <c r="F44">
-        <v>0.7663066954643629</v>
+        <v>0.7676025917926566</v>
       </c>
       <c r="G44">
-        <v>0.824622030237581</v>
+        <v>0.8250539956803455</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -1685,10 +1685,10 @@
         <v>0.7943844492440605</v>
       </c>
       <c r="F45">
-        <v>0.7654427645788338</v>
+        <v>0.7645788336933046</v>
       </c>
       <c r="G45">
-        <v>0.8224622030237581</v>
+        <v>0.8220302375809936</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>

</xml_diff>